<commit_message>
Add data quality report to combine endpoint
</commit_message>
<xml_diff>
--- a/sample_data/Book1.xlsx
+++ b/sample_data/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\DataCombiner\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F46418D-4F9B-4C3A-B864-E47A6F61260E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A84A3F73-1FFC-454F-BC80-53A31FCE846B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{BC4E482F-FCC8-4214-9583-ADCD4B5A37DB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t xml:space="preserve">names </t>
   </si>
@@ -36,19 +36,22 @@
     <t>josh</t>
   </si>
   <si>
-    <t>matthew</t>
-  </si>
-  <si>
     <t>ryan</t>
   </si>
   <si>
-    <t>kai</t>
-  </si>
-  <si>
     <t>y</t>
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>kaihan</t>
+  </si>
+  <si>
+    <t>mark</t>
+  </si>
+  <si>
+    <t>max</t>
   </si>
 </sst>
 </file>
@@ -400,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D691D56-0B36-4A6D-84BF-FAB846E50E1F}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -416,31 +419,36 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add appearance count for merged columns
</commit_message>
<xml_diff>
--- a/sample_data/Book1.xlsx
+++ b/sample_data/Book1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\DataCombiner\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A84A3F73-1FFC-454F-BC80-53A31FCE846B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE910D7-5D86-4106-92CC-39FEB024FAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{BC4E482F-FCC8-4214-9583-ADCD4B5A37DB}"/>
+    <workbookView xWindow="8925" yWindow="5415" windowWidth="28800" windowHeight="15345" xr2:uid="{BC4E482F-FCC8-4214-9583-ADCD4B5A37DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,26 +25,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">names </t>
   </si>
   <si>
-    <t>attend?</t>
-  </si>
-  <si>
     <t>josh</t>
   </si>
   <si>
     <t>ryan</t>
   </si>
   <si>
-    <t>y</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
     <t>kaihan</t>
   </si>
   <si>
@@ -52,6 +43,9 @@
   </si>
   <si>
     <t>max</t>
+  </si>
+  <si>
+    <t>phone</t>
   </si>
 </sst>
 </file>
@@ -411,44 +405,44 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>